<commit_message>
Add second email for Debora Cortazar
</commit_message>
<xml_diff>
--- a/data/contactos.xlsx
+++ b/data/contactos.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C190"/>
+  <dimension ref="A1:C191"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2947,712 +2947,729 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Eleonora</t>
+          <t>Débora</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>Echave</t>
+          <t>Cortazar</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>eleonoraechave@gmail.com</t>
+          <t>deboracortazar@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Mónica</t>
+          <t>Eleonora</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>López</t>
+          <t>Echave</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>secretariaprimaria@institutomurialdo.org</t>
+          <t>eleonoraechave@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>Graciela Ponti</t>
+          <t>Mónica</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>Ponti</t>
+          <t>López</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>gracielaponti0@gmail.com</t>
+          <t>secretariaprimaria@institutomurialdo.org</t>
         </is>
       </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>Paola</t>
+          <t>Graciela Ponti</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>Irusta</t>
+          <t>Ponti</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>plirusta35@gmail.com</t>
+          <t>gracielaponti0@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>Pascual</t>
+          <t>Paola</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>Muscianisi</t>
+          <t>Irusta</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>pascualmuscianisi@gmail.com</t>
+          <t>plirusta35@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>Rolando Pablo Ariel</t>
+          <t>Pascual</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>Tagliaferro</t>
+          <t>Muscianisi</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>rolandotagliaferro@gmail.com</t>
+          <t>pascualmuscianisi@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>María Isabel</t>
+          <t>Rolando Pablo Ariel</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>Arce</t>
+          <t>Tagliaferro</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>mia.bell.ma@gmail.com</t>
+          <t>rolandotagliaferro@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Ruben</t>
+          <t>María Isabel</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>Pellegrini</t>
+          <t>Arce</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>pellegriniruben@hotmail.com</t>
+          <t>mia.bell.ma@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Lorena Paola</t>
+          <t>Ruben</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>Ruiz</t>
+          <t>Pellegrini</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>lruiz1739@gmail.com</t>
+          <t>pellegriniruben@hotmail.com</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Lorena Paola</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Tagliaferro</t>
+          <t>Ruiz</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>davidtaglia@hotmail.com</t>
+          <t>lruiz1739@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>Claudia.</t>
+          <t>David</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>Busto</t>
+          <t>Tagliaferro</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>bclaudian012@gmail.com</t>
+          <t>davidtaglia@hotmail.com</t>
         </is>
       </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>Sergio Omar</t>
+          <t>Claudia.</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>Sandoval</t>
+          <t>Busto</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>sergio.sandoval@cat.edu.ar</t>
+          <t>bclaudian012@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>María Soledad</t>
+          <t>Sergio Omar</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>Rosas Villagra</t>
+          <t>Sandoval</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
         <is>
-          <t>marisolrosas1005@gmail.com</t>
+          <t>sergio.sandoval@cat.edu.ar</t>
         </is>
       </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>Gustavo Alejandro</t>
+          <t>María Soledad</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>Orcellet</t>
+          <t>Rosas Villagra</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>gustavoorcellet@gmail.com</t>
+          <t>marisolrosas1005@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>María Cecilia</t>
+          <t>Gustavo Alejandro</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>Miranda</t>
+          <t>Orcellet</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
         <is>
-          <t>hnamaguiphsf@gmail.com</t>
+          <t>gustavoorcellet@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>Leticia Inés</t>
+          <t>María Cecilia</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>Tulian</t>
+          <t>Miranda</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>letitulian@yahoo.com.ar</t>
+          <t>hnamaguiphsf@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>Adriana Perez</t>
+          <t>Leticia Inés</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>Perez</t>
+          <t>Tulian</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>adrylour29@gmail.com</t>
+          <t>letitulian@yahoo.com.ar</t>
         </is>
       </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>Maria Adriana</t>
+          <t>Adriana Perez</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>Tassin</t>
+          <t>Perez</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
         <is>
-          <t>adriana.tassin@institutomurialdo.org</t>
+          <t>adrylour29@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Mariano</t>
+          <t>Maria Adriana</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>Rizzi</t>
+          <t>Tassin</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>marianorizzi76@gmail.com</t>
+          <t>adriana.tassin@institutomurialdo.org</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>Mauricio</t>
+          <t>Mariano</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>Peña</t>
+          <t>Rizzi</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>mpena@colegioscalabrini.edu.ar</t>
+          <t>marianorizzi76@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Gustavo Ariel</t>
+          <t>Mauricio</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>Castro</t>
+          <t>Peña</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>gcastro@fundacionedison.org.ar</t>
+          <t>mpena@colegioscalabrini.edu.ar</t>
         </is>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Alejandra Carolina</t>
+          <t>Gustavo Ariel</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>Caon</t>
+          <t>Castro</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>alecaon18@gmail.com</t>
+          <t>gcastro@fundacionedison.org.ar</t>
         </is>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>Angela Alejandra</t>
+          <t>Alejandra Carolina</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>Sanchez</t>
+          <t>Caon</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>angisanchez1826@gmail.com</t>
+          <t>alecaon18@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Angela Alejandra</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>Parada</t>
+          <t>Sanchez</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>martinparadaccre@gmail.com</t>
+          <t>angisanchez1826@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Andrea Claudia</t>
+          <t>Martin</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>Calle</t>
+          <t>Parada</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>andreaclaucalleg6972@gmail.com</t>
+          <t>martinparadaccre@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Romina</t>
+          <t>Andrea Claudia</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>Iragorre</t>
+          <t>Calle</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>romiragorre@gmail.com</t>
+          <t>andreaclaucalleg6972@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>María Noelia</t>
+          <t>Romina</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
-          <t>Grando</t>
+          <t>Iragorre</t>
         </is>
       </c>
       <c r="C175" t="inlineStr">
         <is>
-          <t>noegrando@gmail.com</t>
+          <t>romiragorre@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Francisco</t>
+          <t>María Noelia</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>Gallart</t>
+          <t>Grando</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>fgallart@institutomurialdo.org</t>
+          <t>noegrando@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Luciano Exequiel</t>
+          <t>Francisco</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
-          <t>Fernandez</t>
+          <t>Gallart</t>
         </is>
       </c>
       <c r="C177" t="inlineStr">
         <is>
-          <t>lucianoexequielfernandez@gmail.com</t>
+          <t>fgallart@institutomurialdo.org</t>
         </is>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Dario</t>
+          <t>Luciano Exequiel</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Gelves</t>
+          <t>Fernandez</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>dariog@fundacionedison.org.ar</t>
+          <t>lucianoexequielfernandez@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>Adriana Elisa</t>
+          <t>Dario</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>Tissera</t>
+          <t>Gelves</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>atissera@fundacionedison.org.ar</t>
+          <t>dariog@fundacionedison.org.ar</t>
         </is>
       </c>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>Mónica Patricia</t>
+          <t>Adriana Elisa</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>Martínez</t>
+          <t>Tissera</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>mmartinez@fundacionedison.org.ar</t>
+          <t>atissera@fundacionedison.org.ar</t>
         </is>
       </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>Carina Alejandra</t>
+          <t>Mónica Patricia</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>Martinez</t>
+          <t>Martínez</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>carina.m.0402@gmail.com</t>
+          <t>mmartinez@fundacionedison.org.ar</t>
         </is>
       </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>Cecilia Cia</t>
+          <t>Carina Alejandra</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>Cia</t>
+          <t>Martinez</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
         <is>
-          <t>ceciliacia45@gmail.com</t>
+          <t>carina.m.0402@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>Agostina</t>
+          <t>Cecilia Cia</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>Romero</t>
+          <t>Cia</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
         <is>
-          <t>agosromero1993@hotmail.com</t>
+          <t>ceciliacia45@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>Anibal Ceferino</t>
+          <t>Agostina</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>Bustos</t>
+          <t>Romero</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>anibalbustos66@gmail.com</t>
+          <t>agosromero1993@hotmail.com</t>
         </is>
       </c>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>Analía</t>
+          <t>Anibal Ceferino</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>Lorente</t>
+          <t>Bustos</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>analiavivianaprivada@gmail.com</t>
+          <t>anibalbustos66@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>María Elena</t>
+          <t>Analía</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>Armendariz</t>
+          <t>Lorente</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
         <is>
-          <t>maruarmendariz75@gmail.com</t>
+          <t>analiavivianaprivada@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>María Teresa Romina</t>
+          <t>María Elena</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>Moreno</t>
+          <t>Armendariz</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>teremoreno799@gmail.com</t>
+          <t>maruarmendariz75@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Maria Isabel</t>
+          <t>María Teresa Romina</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>Motta</t>
+          <t>Moreno</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>marisitamotta@gmail.com</t>
+          <t>teremoreno799@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Facundo</t>
+          <t>Maria Isabel</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
         <is>
-          <t>Vargas</t>
+          <t>Motta</t>
         </is>
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>facundovargas.uda@gmail.com</t>
+          <t>marisitamotta@gmail.com</t>
         </is>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
+          <t>Facundo</t>
+        </is>
+      </c>
+      <c r="B190" t="inlineStr">
+        <is>
+          <t>Vargas</t>
+        </is>
+      </c>
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>facundovargas.uda@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="191">
+      <c r="A191" t="inlineStr">
+        <is>
           <t>Marita</t>
         </is>
       </c>
-      <c r="B190" t="inlineStr">
+      <c r="B191" t="inlineStr">
         <is>
           <t>Atmat</t>
         </is>
       </c>
-      <c r="C190" t="inlineStr">
+      <c r="C191" t="inlineStr">
         <is>
           <t>amatm@me.com</t>
         </is>

</xml_diff>